<commit_message>
20260928_dbt 배선 2차 완료.
</commit_message>
<xml_diff>
--- a/30_output_share/05_지표GOLD매핑.xlsx
+++ b/30_output_share/05_지표GOLD매핑.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-16 — 본 파일은 자동 생성물입니다. 직접 수정 금지 — 생성기 scripts/gen_metric_gold_mapping.py 수정 후 재실행하세요.</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-28 — 본 파일은 자동 생성물입니다. 직접 수정 금지 — 생성기 scripts/gen_metric_gold_mapping.py 수정 후 재실행하세요.</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-16</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,729/4,716,360 (49.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,458/4,716,088 (49.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,729/4,716,360 (49.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,458/4,716,088 (49.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,729/4,716,360 (49.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,458/4,716,088 (49.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.DEV_CNT` 비영 2,025,238/41,508,842 (4.9%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.DEV_CNT` 비영 2,025,221/41,508,824 (4.9%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.DEV_CNT` 비영 2,025,238/41,508,842 (4.9%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.DEV_CNT` 비영 2,025,221/41,508,824 (4.9%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.AD_COST` 비영 234,859/248,196 (94.6%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_AD_PERFORMANCE.AD_COST` 비영 58,678/77,505 (75.7%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.AD_COST` 비영 234,859/248,196 (94.6%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_AD_PERFORMANCE.AD_COST` 비영 58,678/77,505 (75.7%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.AD_COST` 비영 234,859/248,196 (94.6%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_AD_PERFORMANCE.AD_COST` 비영 58,678/77,505 (75.7%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.CLICKS` 비영 176,578/248,196 (71.1%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_AD_PERFORMANCE.CLICKS` 비영 25,148/77,505 (32.4%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.AGENCY_CONV_MEMBERS` 비영 46,485/248,196 (18.7%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_AD_PERFORMANCE.AGENCY_CONV_MEMBERS` 비영 7,139/77,505 (9.2%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 8,905행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_AD_CREATIVE` 3,367행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.IMPRESSIONS` 비영 199,322/248,196 (80.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_AD_PERFORMANCE.IMPRESSIONS` 비영 23,255/77,505 (30.0%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.CLICKS` 비영 176,578/248,196 (71.1%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_AD_PERFORMANCE.CLICKS` 비영 25,148/77,505 (32.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_AD_PERFORMANCE.INBOUND_CALL` 비영 22,452/248,196 (9.0%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_AD_PERFORMANCE.INBOUND_CALL` 비영 21,459/77,505 (27.7%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,431/4,716,360 (22.5%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,430/4,716,088 (22.5%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -2945,14 +2945,14 @@
           <t>회원번호 기준, 회원상태가 미납인 회원의 총 개발 건 ( = 전체 후원금액 / 10,000 )</t>
         </is>
       </c>
-      <c r="L40" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 비영 3,381,518/41,508,824 (8.1%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -3079,14 +3079,14 @@
           <t>회원번호 기준, 후원사업(세부캠페인)별 총 감액 건 ( = 전체 감액금액 / 10,000 )</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.DECREASE_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.DECREASE_CNT` 비영 115,399/41,508,824 (0.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.MONTH_END_ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.MONTH_END_ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="M50" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.DEV_CNT` 비영 2,025,238/41,508,842 (4.9%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.DEV_CNT` 비영 2,025,221/41,508,824 (4.9%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.YEAR_START_ACTIVE_CNT` 비영 36,847,772/41,508,842 (88.8%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.YEAR_START_ACTIVE_CNT` 비영 36,847,772/41,508,824 (88.8%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -3992,7 +3992,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.MONTH_END_ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.MONTH_END_ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PREV_MONTH_END_ACTIVE_CNT` 비영 39,122,763/41,508,842 (94.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PREV_MONTH_END_ACTIVE_CNT` 비영 39,122,763/41,508,824 (94.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="M58" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4189,7 @@
       </c>
       <c r="M59" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="M60" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,431/4,716,360 (22.5%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,430/4,716,088 (22.5%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="M61" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,431/4,716,360 (22.5%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,430/4,716,088 (22.5%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="M62" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,431/4,716,360 (22.5%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.STOP_CNT` 비영 1,061,430/4,716,088 (22.5%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="M67" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="M68" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="M70" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.REGULAR_FEE` 비영 36,800,958/41,508,842 (88.7%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.REGULAR_FEE` 비영 36,800,958/41,508,824 (88.7%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="M73" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="M74" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="M75" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.BILLED_AMT` 비영 38,579,737/41,508,842 (92.9%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.BILLED_AMT` 비영 38,579,737/41,508,824 (92.9%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5525,14 +5525,14 @@
           <t>미납(건) / 활동(건)</t>
         </is>
       </c>
-      <c r="L80" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M80" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 비영 3,381,518/41,508,824 (8.1%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5592,14 +5592,14 @@
           <t>신규미납(건) / 신규활동(건)</t>
         </is>
       </c>
-      <c r="L81" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L81" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M81" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 비영 3,381,518/41,508,824 (8.1%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5659,14 +5659,14 @@
           <t>기존미납(건) / 기존활동(건)</t>
         </is>
       </c>
-      <c r="L82" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M82" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 비영 3,381,518/41,508,824 (8.1%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -5726,14 +5726,14 @@
           <t>후원사업 미납(건) / 후원사업 활동(건)</t>
         </is>
       </c>
-      <c r="L83" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L83" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M83" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.UNPAID_CNT` 비영 3,381,518/41,508,824 (8.1%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="M89" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MESSAGE_DISPATCH.SEND_MEMBERS` 비영 41,969,590/41,969,590 (100.0%)</t>
+          <t>실측: `FACT_MESSAGE_DISPATCH.SEND_MEMBERS` 비영 41,935,344/41,935,344 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="M90" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MESSAGE_DISPATCH.SUCCESS_MEMBERS` 비영 25,417,305/41,969,590 (60.6%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MESSAGE_DISPATCH.SUCCESS_MEMBERS` 비영 25,384,521/41,935,344 (60.5%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -6253,7 +6253,7 @@
       </c>
       <c r="M91" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MESSAGE_DISPATCH.FAIL_MEMBERS` 비영 2,034,794/41,969,590 (4.8%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MESSAGE_DISPATCH.FAIL_MEMBERS` 비영 2,034,467/41,935,344 (4.9%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -6844,14 +6844,14 @@
         </is>
       </c>
       <c r="K101" s="4" t="inlineStr"/>
-      <c r="L101" s="5" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="L101" s="7" t="inlineStr">
+        <is>
+          <t>WAIT</t>
         </is>
       </c>
       <c r="M101" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_BIGQUERY_BEHAVIOR.SESSION_CNT` 비영 160,166/160,166 (100.0%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_BIGQUERY_BEHAVIOR` **0행** — 테이블 미적재</t>
         </is>
       </c>
     </row>
@@ -6906,7 +6906,7 @@
       </c>
       <c r="M102" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_BIGQUERY_BEHAVIOR.AVG_SESSION_DURATION` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_BIGQUERY_BEHAVIOR` **0행** — 테이블 미적재</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6973,7 @@
       </c>
       <c r="M103" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_BIGQUERY_EVENT` 7,862행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_BIGQUERY_EVENT` 1행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -7040,7 +7040,7 @@
       </c>
       <c r="M104" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_BIGQUERY_EVENT` 7,862행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_BIGQUERY_EVENT` 1행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="M105" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_BIGQUERY_EVENT` 7,862행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_BIGQUERY_EVENT` 1행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -7241,7 +7241,7 @@
       </c>
       <c r="M107" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_BIGQUERY_SOURCE` 142행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_BIGQUERY_SOURCE` 1행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="M108" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_BIGQUERY_SOURCE` 142행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_BIGQUERY_SOURCE` 1행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -7474,14 +7474,14 @@
         </is>
       </c>
       <c r="K111" s="4" t="inlineStr"/>
-      <c r="L111" s="5" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="L111" s="7" t="inlineStr">
+        <is>
+          <t>WAIT</t>
         </is>
       </c>
       <c r="M111" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_BIGQUERY_BEHAVIOR.SCROLL_DEPTH` 비영 30,842/160,166 (19.3%) · ⚠️ 채움률은 **적재된 샤드 내부** 기준이다 — GA4 전기간 미입고(G-5)</t>
+          <t>실측: `FACT_BIGQUERY_BEHAVIOR` **0행** — 테이블 미적재</t>
         </is>
       </c>
     </row>
@@ -7536,7 +7536,7 @@
       </c>
       <c r="M112" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_BIGQUERY_BEHAVIOR.BOUNCE_RATE` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_BIGQUERY_BEHAVIOR` **0행** — 테이블 미적재</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="M113" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_BIGQUERY_SOURCE` 142행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_BIGQUERY_SOURCE` 1행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -9327,7 +9327,7 @@
       </c>
       <c r="M141" s="4" t="inlineStr">
         <is>
-          <t>추정: 배속 차원 `DIM_DATE` 16,437행 실재 — 대응 물리 컬럼 미특정</t>
+          <t>추정: 배속 차원 `DIM_DATE` 73,415행 실재 — 대응 물리 컬럼 미특정</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="M152" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_MEMBERS` 비영 2,325,729/4,716,360 (49.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_MEMBERS` 비영 2,325,458/4,716,088 (49.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -10011,7 +10011,7 @@
       </c>
       <c r="M153" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,729/4,716,360 (49.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_CNT` 비영 2,325,458/4,716,088 (49.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -10067,14 +10067,14 @@
         </is>
       </c>
       <c r="K154" s="4" t="inlineStr"/>
-      <c r="L154" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L154" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M154" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.INCREASE_MEMBERS` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.INCREASE_MEMBERS` 비영 1,840,830/41,508,824 (4.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -10130,14 +10130,14 @@
         </is>
       </c>
       <c r="K155" s="4" t="inlineStr"/>
-      <c r="L155" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L155" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M155" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.INCREASE_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.INCREASE_CNT` 비영 1,840,830/41,508,824 (4.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -10436,7 +10436,7 @@
       </c>
       <c r="M160" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_MEMBERS` 비영 39,854,335/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_MEMBERS` 비영 39,854,330/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -10499,7 +10499,7 @@
       </c>
       <c r="M161" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -10618,14 +10618,14 @@
         </is>
       </c>
       <c r="K163" s="4" t="inlineStr"/>
-      <c r="L163" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L163" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="M163" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CUM_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CUM_CNT` 비영 40,335,569/41,508,824 (97.2%)</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
       </c>
       <c r="M170" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_MEMBERS` 비영 2,325,729/4,716,360 (49.3%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_MEMBERS` 비영 2,325,458/4,716,088 (49.3%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -11495,7 +11495,7 @@
       </c>
       <c r="M177" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -11562,7 +11562,7 @@
       </c>
       <c r="M178" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -11629,7 +11629,7 @@
       </c>
       <c r="M179" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -11696,7 +11696,7 @@
       </c>
       <c r="M180" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,326/41,508,842 (96.0%)</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.ACTIVE_CNT` 비영 39,854,321/41,508,824 (96.0%)</t>
         </is>
       </c>
     </row>
@@ -11763,7 +11763,7 @@
       </c>
       <c r="M181" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -11830,7 +11830,7 @@
       </c>
       <c r="M182" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -11897,7 +11897,7 @@
       </c>
       <c r="M183" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -11964,7 +11964,7 @@
       </c>
       <c r="M184" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12031,7 +12031,7 @@
       </c>
       <c r="M185" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,491/41,508,842 (2.4%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.STOP_CNT` 비영 992,490/41,508,824 (2.4%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12091,14 +12091,14 @@
           <t>후원취소 및 감액한 후원사업의 금액 / 10,000</t>
         </is>
       </c>
-      <c r="L186" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L186" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M186" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.CHURN_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.CHURN_CNT` 비영 1,227,134/41,508,824 (3.0%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12158,14 +12158,14 @@
           <t>캠페인별 이탈(건) / 캠페인별 개발(건)</t>
         </is>
       </c>
-      <c r="L187" s="7" t="inlineStr">
-        <is>
-          <t>WAIT</t>
+      <c r="L187" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M187" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.CHURN_CNT` 전건 0 — 설계O·값 미주입</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.CHURN_CNT` 비영 1,227,134/41,508,824 (3.0%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12232,7 +12232,7 @@
       </c>
       <c r="M188" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12299,7 +12299,7 @@
       </c>
       <c r="M189" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12366,7 +12366,7 @@
       </c>
       <c r="M190" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12433,7 +12433,7 @@
       </c>
       <c r="M191" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="M192" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,842 (90.2%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MEMBER_MONTHLY.PAID_FEE` 비영 37,459,838/41,508,824 (90.2%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12768,7 +12768,7 @@
       </c>
       <c r="M196" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MESSAGE_DISPATCH.SEND_MEMBERS` 비영 41,969,590/41,969,590 (100.0%)</t>
+          <t>실측: `FACT_MESSAGE_DISPATCH.SEND_MEMBERS` 비영 41,935,344/41,935,344 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="M197" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MESSAGE_DISPATCH.SUCCESS_MEMBERS` 비영 25,417,305/41,969,590 (60.6%) · 채움률 95% 미만</t>
+          <t>실측: `FACT_MESSAGE_DISPATCH.SUCCESS_MEMBERS` 비영 25,384,521/41,935,344 (60.5%) · 채움률 95% 미만</t>
         </is>
       </c>
     </row>
@@ -12961,7 +12961,7 @@
       </c>
       <c r="M199" s="4" t="inlineStr">
         <is>
-          <t>실측: `FACT_MEMBER_EVENT.DEV_MEMBERS` 비영 2,325,729/4,716,360 (49.3%) · GA↔CRM identity 커버리지 종속</t>
+          <t>실측: `FACT_MEMBER_EVENT.DEV_MEMBERS` 비영 2,325,458/4,716,088 (49.3%) · GA↔CRM identity 커버리지 종속</t>
         </is>
       </c>
     </row>
@@ -14189,7 +14189,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-16</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -17311,7 +17311,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-16</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-09-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
20261002_mstr반영 및 1차 정리
</commit_message>
<xml_diff>
--- a/30_output_share/05_지표GOLD매핑.xlsx
+++ b/30_output_share/05_지표GOLD매핑.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-01 — 본 파일은 자동 생성물입니다. 직접 수정 금지 — 생성기 scripts/gen_metric_gold_mapping.py 수정 후 재실행하세요.</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-02 — 본 파일은 자동 생성물입니다. 직접 수정 금지 — 생성기 scripts/gen_metric_gold_mapping.py 수정 후 재실행하세요.</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-01</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -14205,7 +14205,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-01</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -17327,7 +17327,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-01</t>
+          <t>⚙️ 생성기: scripts/gen_metric_gold_mapping.py · 측정일 2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>